<commit_message>
Final version time series
</commit_message>
<xml_diff>
--- a/data/expClassification.xlsx
+++ b/data/expClassification.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/f215465b21b5e6e2/Studium/34_Github/PrediKit/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9B367332-FB0E-409F-8512-C6A46E4CD7DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="7" documentId="8_{9B367332-FB0E-409F-8512-C6A46E4CD7DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EA8EEE4C-FC60-451C-87A4-1D4E5A45BAF7}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="3" xr2:uid="{3FCB8BB5-2836-44B8-913B-2365A2F1C054}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="1" xr2:uid="{3FCB8BB5-2836-44B8-913B-2365A2F1C054}"/>
   </bookViews>
   <sheets>
     <sheet name="readme" sheetId="4" r:id="rId1"/>
@@ -50,15 +50,6 @@
     <t>y</t>
   </si>
   <si>
-    <t>X1</t>
-  </si>
-  <si>
-    <t>X2</t>
-  </si>
-  <si>
-    <t>X3</t>
-  </si>
-  <si>
     <t>Author</t>
   </si>
   <si>
@@ -71,7 +62,16 @@
     <t>Version</t>
   </si>
   <si>
-    <t>X4</t>
+    <t>sepal_length</t>
+  </si>
+  <si>
+    <t>sepal_width</t>
+  </si>
+  <si>
+    <t>petal_length</t>
+  </si>
+  <si>
+    <t>petal_width</t>
   </si>
 </sst>
 </file>
@@ -124,10 +124,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -470,15 +471,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="B1" t="s">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="B2" s="2">
         <v>46250</v>
@@ -486,7 +487,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="B3">
         <v>0.1</v>
@@ -506,16 +507,16 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="B1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>9</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -2936,16 +2937,16 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="B1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>9</v>
       </c>
       <c r="F1" s="1" t="s">
@@ -3566,16 +3567,16 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E1" s="1" t="s">
+      <c r="B1" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>9</v>
       </c>
       <c r="F1" s="1" t="s">

</xml_diff>